<commit_message>
feat: Refatora tratamento de métricas e melhora os cálculos estatísticos no OptimizerGym
</commit_message>
<xml_diff>
--- a/templates/template_objective_table.xlsx
+++ b/templates/template_objective_table.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Recompensas" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="43">
   <si>
     <t xml:space="preserve">Cenário</t>
   </si>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t xml:space="preserve">Minimizar o tempo de entrega dos motoristas a partir do tempo efetivo gasto (Com penalização 5x para pedidos não coletados) ao final do episódio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objetivo 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximizar o número de pedidos entregues Recompensa positiva a cada pedido entregue</t>
   </si>
 </sst>
 </file>
@@ -640,7 +646,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="33.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="42.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="0" width="27.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2299,9 +2305,158 @@
       <c r="AB42" s="30"/>
       <c r="AC42" s="30"/>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" s="9"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="10"/>
+      <c r="U43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="V43" s="9"/>
+      <c r="W43" s="10"/>
+      <c r="X43" s="10"/>
+      <c r="Y43" s="10"/>
+      <c r="Z43" s="10"/>
+      <c r="AA43" s="10"/>
+      <c r="AB43" s="10"/>
+      <c r="AC43" s="10"/>
+    </row>
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="M44" s="13"/>
+      <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
+      <c r="P44" s="13"/>
+      <c r="Q44" s="13"/>
+      <c r="R44" s="13"/>
+      <c r="S44" s="13"/>
+      <c r="T44" s="13"/>
+      <c r="U44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="V44" s="13"/>
+      <c r="W44" s="13"/>
+      <c r="X44" s="13"/>
+      <c r="Y44" s="13"/>
+      <c r="Z44" s="13"/>
+      <c r="AA44" s="13"/>
+      <c r="AB44" s="13"/>
+      <c r="AC44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M45" s="27"/>
+      <c r="N45" s="28"/>
+      <c r="O45" s="28"/>
+      <c r="P45" s="27"/>
+      <c r="Q45" s="17"/>
+      <c r="R45" s="17"/>
+      <c r="S45" s="17"/>
+      <c r="T45" s="17"/>
+      <c r="U45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="V45" s="27"/>
+      <c r="W45" s="28"/>
+      <c r="X45" s="28"/>
+      <c r="Y45" s="27"/>
+      <c r="Z45" s="17"/>
+      <c r="AA45" s="17"/>
+      <c r="AB45" s="17"/>
+      <c r="AC45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="30"/>
+      <c r="E46" s="30"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="M46" s="30"/>
+      <c r="N46" s="30"/>
+      <c r="O46" s="30"/>
+      <c r="P46" s="30"/>
+      <c r="Q46" s="30"/>
+      <c r="R46" s="30"/>
+      <c r="S46" s="30"/>
+      <c r="T46" s="30"/>
+      <c r="U46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="V46" s="30"/>
+      <c r="W46" s="30"/>
+      <c r="X46" s="30"/>
+      <c r="Y46" s="30"/>
+      <c r="Z46" s="30"/>
+      <c r="AA46" s="30"/>
+      <c r="AB46" s="30"/>
+      <c r="AC46" s="30"/>
+    </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3257,7 +3412,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="25">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -3281,6 +3436,8 @@
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="A39:A42"/>
     <mergeCell ref="B39:B42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="B43:B46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3325,7 +3482,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="33.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="42.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="0" width="27.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4984,9 +5141,158 @@
       <c r="AB42" s="30"/>
       <c r="AC42" s="30"/>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" s="9"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="10"/>
+      <c r="U43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="V43" s="9"/>
+      <c r="W43" s="10"/>
+      <c r="X43" s="10"/>
+      <c r="Y43" s="10"/>
+      <c r="Z43" s="10"/>
+      <c r="AA43" s="10"/>
+      <c r="AB43" s="10"/>
+      <c r="AC43" s="10"/>
+    </row>
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="M44" s="13"/>
+      <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
+      <c r="P44" s="13"/>
+      <c r="Q44" s="13"/>
+      <c r="R44" s="13"/>
+      <c r="S44" s="13"/>
+      <c r="T44" s="13"/>
+      <c r="U44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="V44" s="13"/>
+      <c r="W44" s="13"/>
+      <c r="X44" s="13"/>
+      <c r="Y44" s="13"/>
+      <c r="Z44" s="13"/>
+      <c r="AA44" s="13"/>
+      <c r="AB44" s="13"/>
+      <c r="AC44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M45" s="27"/>
+      <c r="N45" s="28"/>
+      <c r="O45" s="28"/>
+      <c r="P45" s="27"/>
+      <c r="Q45" s="17"/>
+      <c r="R45" s="17"/>
+      <c r="S45" s="17"/>
+      <c r="T45" s="17"/>
+      <c r="U45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="V45" s="27"/>
+      <c r="W45" s="28"/>
+      <c r="X45" s="28"/>
+      <c r="Y45" s="27"/>
+      <c r="Z45" s="17"/>
+      <c r="AA45" s="17"/>
+      <c r="AB45" s="17"/>
+      <c r="AC45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="30"/>
+      <c r="E46" s="30"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="M46" s="30"/>
+      <c r="N46" s="30"/>
+      <c r="O46" s="30"/>
+      <c r="P46" s="30"/>
+      <c r="Q46" s="30"/>
+      <c r="R46" s="30"/>
+      <c r="S46" s="30"/>
+      <c r="T46" s="30"/>
+      <c r="U46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="V46" s="30"/>
+      <c r="W46" s="30"/>
+      <c r="X46" s="30"/>
+      <c r="Y46" s="30"/>
+      <c r="Z46" s="30"/>
+      <c r="AA46" s="30"/>
+      <c r="AB46" s="30"/>
+      <c r="AC46" s="30"/>
+    </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5942,7 +6248,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="25">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -5966,6 +6272,8 @@
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="A39:A42"/>
     <mergeCell ref="B39:B42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="B43:B46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6010,7 +6318,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="33.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="42.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="27" style="0" width="27.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="31.32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7669,9 +7977,158 @@
       <c r="AB42" s="30"/>
       <c r="AC42" s="30"/>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" s="9"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="10"/>
+      <c r="U43" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="V43" s="9"/>
+      <c r="W43" s="10"/>
+      <c r="X43" s="10"/>
+      <c r="Y43" s="10"/>
+      <c r="Z43" s="10"/>
+      <c r="AA43" s="10"/>
+      <c r="AB43" s="10"/>
+      <c r="AC43" s="10"/>
+    </row>
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="13"/>
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="13"/>
+      <c r="J44" s="13"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="M44" s="13"/>
+      <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
+      <c r="P44" s="13"/>
+      <c r="Q44" s="13"/>
+      <c r="R44" s="13"/>
+      <c r="S44" s="13"/>
+      <c r="T44" s="13"/>
+      <c r="U44" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="V44" s="13"/>
+      <c r="W44" s="13"/>
+      <c r="X44" s="13"/>
+      <c r="Y44" s="13"/>
+      <c r="Z44" s="13"/>
+      <c r="AA44" s="13"/>
+      <c r="AB44" s="13"/>
+      <c r="AC44" s="13"/>
+    </row>
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M45" s="27"/>
+      <c r="N45" s="28"/>
+      <c r="O45" s="28"/>
+      <c r="P45" s="27"/>
+      <c r="Q45" s="17"/>
+      <c r="R45" s="17"/>
+      <c r="S45" s="17"/>
+      <c r="T45" s="17"/>
+      <c r="U45" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="V45" s="27"/>
+      <c r="W45" s="28"/>
+      <c r="X45" s="28"/>
+      <c r="Y45" s="27"/>
+      <c r="Z45" s="17"/>
+      <c r="AA45" s="17"/>
+      <c r="AB45" s="17"/>
+      <c r="AC45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="30"/>
+      <c r="E46" s="30"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30"/>
+      <c r="K46" s="30"/>
+      <c r="L46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="M46" s="30"/>
+      <c r="N46" s="30"/>
+      <c r="O46" s="30"/>
+      <c r="P46" s="30"/>
+      <c r="Q46" s="30"/>
+      <c r="R46" s="30"/>
+      <c r="S46" s="30"/>
+      <c r="T46" s="30"/>
+      <c r="U46" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="V46" s="30"/>
+      <c r="W46" s="30"/>
+      <c r="X46" s="30"/>
+      <c r="Y46" s="30"/>
+      <c r="Z46" s="30"/>
+      <c r="AA46" s="30"/>
+      <c r="AB46" s="30"/>
+      <c r="AC46" s="30"/>
+    </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8627,7 +9084,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="25">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -8651,6 +9108,8 @@
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="A39:A42"/>
     <mergeCell ref="B39:B42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="B43:B46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
fix: Corrige nomenclatura da variável de tempo de decisão no ambiente de simulação
</commit_message>
<xml_diff>
--- a/templates/template_objective_table.xlsx
+++ b/templates/template_objective_table.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Recompensas" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Tempo Efetivo Gasto" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Distância Percorrida" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Recompensas" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Tempo Efetivo Gasto" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Distância Percorrida" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="47">
   <si>
     <t xml:space="preserve">Cenário</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t xml:space="preserve">Penaliza pelo tempo total de cada pedido entregue neste step. Quanto mais rápido o pedido for entregue, menor a penalidade (maior a recompensa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objetivo 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penaliza pelo tempo gasto de cada pedido que está na pipeline de entrega (pedidos prontos e não entregues) e de cada pedido entregue neste step. </t>
   </si>
 </sst>
 </file>
@@ -623,119 +629,13 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC1000"/>
-  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -2725,10 +2625,158 @@
       <c r="AB50" s="31"/>
       <c r="AC50" s="31"/>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="10"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11"/>
+      <c r="K51" s="11"/>
+      <c r="L51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="M51" s="10"/>
+      <c r="N51" s="11"/>
+      <c r="O51" s="11"/>
+      <c r="P51" s="11"/>
+      <c r="Q51" s="11"/>
+      <c r="R51" s="11"/>
+      <c r="S51" s="11"/>
+      <c r="T51" s="11"/>
+      <c r="U51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="V51" s="10"/>
+      <c r="W51" s="11"/>
+      <c r="X51" s="11"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="11"/>
+      <c r="AA51" s="11"/>
+      <c r="AB51" s="11"/>
+      <c r="AC51" s="11"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+      <c r="T52" s="14"/>
+      <c r="U52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="V52" s="14"/>
+      <c r="W52" s="14"/>
+      <c r="X52" s="14"/>
+      <c r="Y52" s="14"/>
+      <c r="Z52" s="14"/>
+      <c r="AA52" s="14"/>
+      <c r="AB52" s="14"/>
+      <c r="AC52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="28"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="28"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="M53" s="28"/>
+      <c r="N53" s="29"/>
+      <c r="O53" s="29"/>
+      <c r="P53" s="28"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="18"/>
+      <c r="U53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="V53" s="28"/>
+      <c r="W53" s="29"/>
+      <c r="X53" s="29"/>
+      <c r="Y53" s="28"/>
+      <c r="Z53" s="18"/>
+      <c r="AA53" s="18"/>
+      <c r="AB53" s="18"/>
+      <c r="AC53" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" s="31"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="31"/>
+      <c r="J54" s="31"/>
+      <c r="K54" s="31"/>
+      <c r="L54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="M54" s="31"/>
+      <c r="N54" s="31"/>
+      <c r="O54" s="31"/>
+      <c r="P54" s="31"/>
+      <c r="Q54" s="31"/>
+      <c r="R54" s="31"/>
+      <c r="S54" s="31"/>
+      <c r="T54" s="31"/>
+      <c r="U54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="V54" s="31"/>
+      <c r="W54" s="31"/>
+      <c r="X54" s="31"/>
+      <c r="Y54" s="31"/>
+      <c r="Z54" s="31"/>
+      <c r="AA54" s="31"/>
+      <c r="AB54" s="31"/>
+      <c r="AC54" s="31"/>
+    </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3676,7 +3724,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -3704,6 +3752,8 @@
     <mergeCell ref="B43:B46"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B54"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3716,12 +3766,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC1000"/>
-  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -5711,10 +5761,158 @@
       <c r="AB50" s="31"/>
       <c r="AC50" s="31"/>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="10"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11"/>
+      <c r="K51" s="11"/>
+      <c r="L51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="M51" s="10"/>
+      <c r="N51" s="11"/>
+      <c r="O51" s="11"/>
+      <c r="P51" s="11"/>
+      <c r="Q51" s="11"/>
+      <c r="R51" s="11"/>
+      <c r="S51" s="11"/>
+      <c r="T51" s="11"/>
+      <c r="U51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="V51" s="10"/>
+      <c r="W51" s="11"/>
+      <c r="X51" s="11"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="11"/>
+      <c r="AA51" s="11"/>
+      <c r="AB51" s="11"/>
+      <c r="AC51" s="11"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+      <c r="T52" s="14"/>
+      <c r="U52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="V52" s="14"/>
+      <c r="W52" s="14"/>
+      <c r="X52" s="14"/>
+      <c r="Y52" s="14"/>
+      <c r="Z52" s="14"/>
+      <c r="AA52" s="14"/>
+      <c r="AB52" s="14"/>
+      <c r="AC52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="28"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="28"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="M53" s="28"/>
+      <c r="N53" s="29"/>
+      <c r="O53" s="29"/>
+      <c r="P53" s="28"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="18"/>
+      <c r="U53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="V53" s="28"/>
+      <c r="W53" s="29"/>
+      <c r="X53" s="29"/>
+      <c r="Y53" s="28"/>
+      <c r="Z53" s="18"/>
+      <c r="AA53" s="18"/>
+      <c r="AB53" s="18"/>
+      <c r="AC53" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" s="31"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="31"/>
+      <c r="J54" s="31"/>
+      <c r="K54" s="31"/>
+      <c r="L54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="M54" s="31"/>
+      <c r="N54" s="31"/>
+      <c r="O54" s="31"/>
+      <c r="P54" s="31"/>
+      <c r="Q54" s="31"/>
+      <c r="R54" s="31"/>
+      <c r="S54" s="31"/>
+      <c r="T54" s="31"/>
+      <c r="U54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="V54" s="31"/>
+      <c r="W54" s="31"/>
+      <c r="X54" s="31"/>
+      <c r="Y54" s="31"/>
+      <c r="Z54" s="31"/>
+      <c r="AA54" s="31"/>
+      <c r="AB54" s="31"/>
+      <c r="AC54" s="31"/>
+    </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6662,7 +6860,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -6690,6 +6888,8 @@
     <mergeCell ref="B43:B46"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B54"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6702,12 +6902,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC1000"/>
-  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.63671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -8697,10 +8897,158 @@
       <c r="AB50" s="31"/>
       <c r="AC50" s="31"/>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="10"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="11"/>
+      <c r="K51" s="11"/>
+      <c r="L51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="M51" s="10"/>
+      <c r="N51" s="11"/>
+      <c r="O51" s="11"/>
+      <c r="P51" s="11"/>
+      <c r="Q51" s="11"/>
+      <c r="R51" s="11"/>
+      <c r="S51" s="11"/>
+      <c r="T51" s="11"/>
+      <c r="U51" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="V51" s="10"/>
+      <c r="W51" s="11"/>
+      <c r="X51" s="11"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="11"/>
+      <c r="AA51" s="11"/>
+      <c r="AB51" s="11"/>
+      <c r="AC51" s="11"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="14"/>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="14"/>
+      <c r="P52" s="14"/>
+      <c r="Q52" s="14"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="14"/>
+      <c r="T52" s="14"/>
+      <c r="U52" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="V52" s="14"/>
+      <c r="W52" s="14"/>
+      <c r="X52" s="14"/>
+      <c r="Y52" s="14"/>
+      <c r="Z52" s="14"/>
+      <c r="AA52" s="14"/>
+      <c r="AB52" s="14"/>
+      <c r="AC52" s="14"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="28"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="28"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="M53" s="28"/>
+      <c r="N53" s="29"/>
+      <c r="O53" s="29"/>
+      <c r="P53" s="28"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="18"/>
+      <c r="U53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="V53" s="28"/>
+      <c r="W53" s="29"/>
+      <c r="X53" s="29"/>
+      <c r="Y53" s="28"/>
+      <c r="Z53" s="18"/>
+      <c r="AA53" s="18"/>
+      <c r="AB53" s="18"/>
+      <c r="AC53" s="18"/>
+    </row>
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" s="31"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="31"/>
+      <c r="J54" s="31"/>
+      <c r="K54" s="31"/>
+      <c r="L54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="M54" s="31"/>
+      <c r="N54" s="31"/>
+      <c r="O54" s="31"/>
+      <c r="P54" s="31"/>
+      <c r="Q54" s="31"/>
+      <c r="R54" s="31"/>
+      <c r="S54" s="31"/>
+      <c r="T54" s="31"/>
+      <c r="U54" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="V54" s="31"/>
+      <c r="W54" s="31"/>
+      <c r="X54" s="31"/>
+      <c r="Y54" s="31"/>
+      <c r="Z54" s="31"/>
+      <c r="AA54" s="31"/>
+      <c r="AB54" s="31"/>
+      <c r="AC54" s="31"/>
+    </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -9648,7 +9996,7 @@
     <row r="999" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
     <mergeCell ref="D1:K1"/>
     <mergeCell ref="M1:T1"/>
     <mergeCell ref="V1:AC1"/>
@@ -9676,6 +10024,8 @@
     <mergeCell ref="B43:B46"/>
     <mergeCell ref="A47:A50"/>
     <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B54"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.511805555555556" right="0.511805555555556" top="0.7875" bottom="0.7875" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>